<commit_message>
refactor: salvando alteraçõs de validação
</commit_message>
<xml_diff>
--- a/Tabela de Pessoas.xlsx
+++ b/Tabela de Pessoas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="1" min="3" max="3"/>
@@ -2569,6 +2569,189 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>joana P Santos</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>11912345678</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>25</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>dsdh@gmm.com.br</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>06666000</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Mario Veloso Serqueira</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>43</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Carlos Drummord Andrade</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Caracas</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>joão P Santos</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>912345678</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>25</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>dsdh@gmm.com.br</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>06666000</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Mario Veloso Serqueira</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>43</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Carlos Drummord Andrade</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Caracas</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>sdjsghjagsdja</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>098765432</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>65</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>jhgasdgj@sahdkjfkhf.com</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>09876-543</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ghghjshjffahgfhjaf</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>343</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>hjsgfhs</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>kjshdjfhs</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>ds</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>